<commit_message>
fix: working on the demo
</commit_message>
<xml_diff>
--- a/Program.xlsx
+++ b/Program.xlsx
@@ -5,17 +5,18 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://liveunibo-my.sharepoint.com/personal/matteo_francia2_studio_unibo_it/Documents/teaching-bigdata/AA2526-unibo-bigdataandcloudplatforms/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\repos\teaching\AA2627-unibo-bdcp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="147" documentId="13_ncr:1_{F7F973B8-4F16-4EF1-8487-709103825833}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9F35B8B1-6749-4F8D-97CC-8EC8714A263F}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{64E5802E-1FE7-403E-B8D1-DB4620768C4F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="57480" yWindow="15990" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="46296" windowHeight="25416" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="AA2526" sheetId="3" r:id="rId1"/>
-    <sheet name="AA2425" sheetId="2" r:id="rId2"/>
-    <sheet name="AA2223" sheetId="1" r:id="rId3"/>
+    <sheet name="AA2627" sheetId="4" r:id="rId1"/>
+    <sheet name="AA2526" sheetId="3" r:id="rId2"/>
+    <sheet name="AA2425" sheetId="2" r:id="rId3"/>
+    <sheet name="AA2223" sheetId="1" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -39,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="217" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="276" uniqueCount="73">
   <si>
     <t>When</t>
   </si>
@@ -252,6 +253,12 @@
   </si>
   <si>
     <t>TOT</t>
+  </si>
+  <si>
+    <t>AULA 2.7, 2h (13-15)</t>
+  </si>
+  <si>
+    <t>Towards data platforms (until lakehouse)</t>
   </si>
 </sst>
 </file>
@@ -471,7 +478,14 @@
     <cellStyle name="Collegamento ipertestuale" xfId="1" builtinId="8"/>
     <cellStyle name="Normale" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="3">
+  <dxfs count="4">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <fill>
         <patternFill>
@@ -768,21 +782,21 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5DE48BDE-AF85-4F5A-91B1-CBAD698B62C1}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{778FCF00-0ED4-4EAC-A0A8-DD346D8625F0}">
   <dimension ref="A1:H23"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="10.81640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.77734375" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="9" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="17.7265625" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="6.7265625" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="8.26953125" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="66.81640625" style="13" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="5.26953125" customWidth="1"/>
-    <col min="8" max="8" width="8.7265625" customWidth="1"/>
+    <col min="3" max="3" width="17.77734375" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="6.77734375" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="8.21875" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="66.77734375" style="13" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="5.21875" customWidth="1"/>
+    <col min="8" max="8" width="8.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -808,16 +822,16 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A2" s="4">
-        <v>45937</v>
+        <v>45942</v>
       </c>
       <c r="B2" s="23">
         <f>WEEKDAY(A2)-1</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>8</v>
+        <v>71</v>
       </c>
       <c r="D2" s="4" t="s">
         <v>9</v>
@@ -833,43 +847,42 @@
         <v>6.6666666666666666E-2</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" s="4">
-        <f>A2</f>
-        <v>45937</v>
+        <v>45943</v>
       </c>
       <c r="B3" s="23">
         <f t="shared" ref="B3:B21" si="0">WEEKDAY(A3)-1</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C3" s="7" t="s">
         <v>11</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="E3" s="22">
         <v>2</v>
       </c>
       <c r="F3" s="13" t="s">
-        <v>12</v>
+        <v>72</v>
       </c>
       <c r="G3" s="22">
         <f>SUM($E$2:E3)/$E$23</f>
         <v>0.13333333333333333</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A4" s="4">
-        <f>A3+7</f>
-        <v>45944</v>
+        <f>A2+7</f>
+        <v>45949</v>
       </c>
       <c r="B4" s="23">
         <f t="shared" si="0"/>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>11</v>
+        <v>71</v>
       </c>
       <c r="D4" s="3" t="s">
         <v>9</v>
@@ -886,14 +899,14 @@
       </c>
       <c r="H4" s="18"/>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A5" s="4">
-        <f>A4+7</f>
-        <v>45951</v>
+        <f>A3+7</f>
+        <v>45950</v>
       </c>
       <c r="B5" s="23">
         <f t="shared" si="0"/>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C5" s="7" t="s">
         <v>11</v>
@@ -912,17 +925,17 @@
         <v>0.26666666666666666</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6" s="4">
-        <f>A5+7</f>
-        <v>45958</v>
+        <f t="shared" ref="A6:A17" si="1">A4+7</f>
+        <v>45956</v>
       </c>
       <c r="B6" s="23">
         <f t="shared" si="0"/>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>8</v>
+        <v>71</v>
       </c>
       <c r="D6" s="4" t="s">
         <v>9</v>
@@ -938,14 +951,14 @@
         <v>0.33333333333333331</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A7" s="4">
-        <f>A6</f>
-        <v>45958</v>
+        <f t="shared" si="1"/>
+        <v>45957</v>
       </c>
       <c r="B7" s="23">
         <f t="shared" si="0"/>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C7" s="7" t="s">
         <v>11</v>
@@ -964,17 +977,17 @@
         <v>0.4</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A8" s="4">
-        <f>A7+7</f>
-        <v>45965</v>
+        <f t="shared" si="1"/>
+        <v>45963</v>
       </c>
       <c r="B8" s="23">
         <f t="shared" si="0"/>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>8</v>
+        <v>71</v>
       </c>
       <c r="D8" s="4" t="s">
         <v>9</v>
@@ -990,14 +1003,14 @@
         <v>0.46666666666666667</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A9" s="4">
-        <f>A8</f>
-        <v>45965</v>
+        <f t="shared" si="1"/>
+        <v>45964</v>
       </c>
       <c r="B9" s="23">
         <f t="shared" si="0"/>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C9" s="7" t="s">
         <v>11</v>
@@ -1016,17 +1029,17 @@
         <v>0.53333333333333333</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A10" s="4">
-        <f>A9+7</f>
-        <v>45972</v>
+        <f t="shared" si="1"/>
+        <v>45970</v>
       </c>
       <c r="B10" s="23">
         <f t="shared" si="0"/>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>8</v>
+        <v>71</v>
       </c>
       <c r="D10" s="4" t="s">
         <v>9</v>
@@ -1042,14 +1055,14 @@
         <v>0.6</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A11" s="4">
-        <f>A10</f>
-        <v>45972</v>
+        <f t="shared" si="1"/>
+        <v>45971</v>
       </c>
       <c r="B11" s="23">
         <f t="shared" si="0"/>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C11" s="7" t="s">
         <v>11</v>
@@ -1068,17 +1081,17 @@
         <v>0.66666666666666663</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A12" s="4">
-        <f>A11+7</f>
-        <v>45979</v>
+        <f t="shared" si="1"/>
+        <v>45977</v>
       </c>
       <c r="B12" s="23">
         <f t="shared" si="0"/>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>8</v>
+        <v>71</v>
       </c>
       <c r="D12" s="4" t="s">
         <v>9</v>
@@ -1089,14 +1102,14 @@
         <v>0.66666666666666663</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A13" s="4">
-        <f>A12</f>
-        <v>45979</v>
+        <f t="shared" si="1"/>
+        <v>45978</v>
       </c>
       <c r="B13" s="23">
         <f t="shared" si="0"/>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C13" s="7" t="s">
         <v>11</v>
@@ -1115,20 +1128,20 @@
         <v>0.73333333333333328</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A14" s="4">
-        <f>A13+7</f>
-        <v>45986</v>
+        <f t="shared" si="1"/>
+        <v>45984</v>
       </c>
       <c r="B14" s="23">
         <f t="shared" si="0"/>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C14" s="7" t="s">
-        <v>8</v>
-      </c>
-      <c r="D14" s="14" t="s">
-        <v>22</v>
+        <v>71</v>
+      </c>
+      <c r="D14" s="4" t="s">
+        <v>9</v>
       </c>
       <c r="E14" s="22">
         <v>2</v>
@@ -1141,20 +1154,20 @@
         <v>0.8</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A15" s="4">
-        <f>A14</f>
-        <v>45986</v>
+        <f t="shared" si="1"/>
+        <v>45985</v>
       </c>
       <c r="B15" s="23">
         <f t="shared" si="0"/>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="D15" s="14" t="s">
-        <v>22</v>
+        <v>11</v>
+      </c>
+      <c r="D15" s="4" t="s">
+        <v>14</v>
       </c>
       <c r="E15" s="22">
         <v>2</v>
@@ -1165,20 +1178,20 @@
         <v>0.8666666666666667</v>
       </c>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A16" s="4">
-        <f>A15+7</f>
-        <v>45993</v>
+        <f t="shared" si="1"/>
+        <v>45991</v>
       </c>
       <c r="B16" s="23">
         <f t="shared" si="0"/>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C16" s="7" t="s">
-        <v>8</v>
-      </c>
-      <c r="D16" s="14" t="s">
-        <v>22</v>
+        <v>71</v>
+      </c>
+      <c r="D16" s="4" t="s">
+        <v>9</v>
       </c>
       <c r="E16" s="22">
         <v>2</v>
@@ -1191,20 +1204,20 @@
         <v>0.93333333333333335</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A17" s="4">
-        <f>A16</f>
-        <v>45993</v>
+        <f t="shared" si="1"/>
+        <v>45992</v>
       </c>
       <c r="B17" s="23">
         <f t="shared" si="0"/>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C17" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="D17" s="14" t="s">
-        <v>22</v>
+      <c r="D17" s="4" t="s">
+        <v>14</v>
       </c>
       <c r="E17" s="22">
         <v>2</v>
@@ -1215,14 +1228,14 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A18" s="4">
         <f>A17+7</f>
-        <v>46000</v>
+        <v>45999</v>
       </c>
       <c r="B18" s="23">
         <f t="shared" si="0"/>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C18" s="7" t="s">
         <v>8</v>
@@ -1232,14 +1245,14 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A19" s="4">
         <f>A18</f>
-        <v>46000</v>
+        <v>45999</v>
       </c>
       <c r="B19" s="23">
         <f t="shared" si="0"/>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C19" s="7" t="s">
         <v>11</v>
@@ -1250,34 +1263,34 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A20" s="4">
         <f>A19+7</f>
-        <v>46007</v>
+        <v>46006</v>
       </c>
       <c r="B20" s="23">
         <f t="shared" si="0"/>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C20" s="7" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="21" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A21" s="4">
         <f>A20</f>
-        <v>46007</v>
+        <v>46006</v>
       </c>
       <c r="B21" s="23">
         <f t="shared" si="0"/>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C21" s="7" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="D22" s="1" t="s">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="D22" s="2" t="s">
         <v>26</v>
       </c>
       <c r="E22" s="2">
@@ -1285,8 +1298,8 @@
         <v>30</v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="D23" s="1" t="s">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="D23" s="2" t="s">
         <v>27</v>
       </c>
       <c r="E23" s="1">
@@ -1311,7 +1324,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F1 E23 D23:D1048576 D19 D1:D17">
-    <cfRule type="cellIs" dxfId="2" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="0" priority="2" operator="equal">
       <formula>"Theory"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -1321,23 +1334,576 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5DE48BDE-AF85-4F5A-91B1-CBAD698B62C1}">
+  <dimension ref="A1:H23"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="10.77734375" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.77734375" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="6.77734375" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="8.21875" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="66.77734375" style="13" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="5.21875" customWidth="1"/>
+    <col min="8" max="8" width="8.77734375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="15" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="21" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A2" s="4">
+        <v>45937</v>
+      </c>
+      <c r="B2" s="23">
+        <f>WEEKDAY(A2)-1</f>
+        <v>2</v>
+      </c>
+      <c r="C2" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="E2" s="22">
+        <v>2</v>
+      </c>
+      <c r="F2" s="13" t="s">
+        <v>10</v>
+      </c>
+      <c r="G2" s="22">
+        <f>SUM($E$2:E2)/$E$23</f>
+        <v>6.6666666666666666E-2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3" s="4">
+        <f>A2</f>
+        <v>45937</v>
+      </c>
+      <c r="B3" s="23">
+        <f t="shared" ref="B3:B21" si="0">WEEKDAY(A3)-1</f>
+        <v>2</v>
+      </c>
+      <c r="C3" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="E3" s="22">
+        <v>2</v>
+      </c>
+      <c r="F3" s="13" t="s">
+        <v>12</v>
+      </c>
+      <c r="G3" s="22">
+        <f>SUM($E$2:E3)/$E$23</f>
+        <v>0.13333333333333333</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A4" s="4">
+        <f>A3+7</f>
+        <v>45944</v>
+      </c>
+      <c r="B4" s="23">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+      <c r="C4" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E4" s="22">
+        <v>2</v>
+      </c>
+      <c r="F4" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="G4" s="22">
+        <f>SUM($E$2:E4)/$E$23</f>
+        <v>0.2</v>
+      </c>
+      <c r="H4" s="18"/>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A5" s="4">
+        <f>A4+7</f>
+        <v>45951</v>
+      </c>
+      <c r="B5" s="23">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="E5" s="22">
+        <v>2</v>
+      </c>
+      <c r="F5" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="G5" s="22">
+        <f>SUM($E$2:E5)/$E$23</f>
+        <v>0.26666666666666666</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A6" s="4">
+        <f>A5+7</f>
+        <v>45958</v>
+      </c>
+      <c r="B6" s="23">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+      <c r="C6" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="E6" s="22">
+        <v>2</v>
+      </c>
+      <c r="F6" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="G6" s="22">
+        <f>SUM($E$2:E6)/$E$23</f>
+        <v>0.33333333333333331</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A7" s="4">
+        <f>A6</f>
+        <v>45958</v>
+      </c>
+      <c r="B7" s="23">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+      <c r="C7" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="E7" s="22">
+        <v>2</v>
+      </c>
+      <c r="F7" s="13" t="s">
+        <v>17</v>
+      </c>
+      <c r="G7" s="22">
+        <f>SUM($E$2:E7)/$E$23</f>
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A8" s="4">
+        <f>A7+7</f>
+        <v>45965</v>
+      </c>
+      <c r="B8" s="23">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+      <c r="C8" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="E8" s="22">
+        <v>2</v>
+      </c>
+      <c r="F8" s="13" t="s">
+        <v>18</v>
+      </c>
+      <c r="G8" s="22">
+        <f>SUM($E$2:E8)/$E$23</f>
+        <v>0.46666666666666667</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A9" s="4">
+        <f>A8</f>
+        <v>45965</v>
+      </c>
+      <c r="B9" s="23">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+      <c r="C9" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="E9" s="22">
+        <v>2</v>
+      </c>
+      <c r="F9" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="G9" s="22">
+        <f>SUM($E$2:E9)/$E$23</f>
+        <v>0.53333333333333333</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A10" s="4">
+        <f>A9+7</f>
+        <v>45972</v>
+      </c>
+      <c r="B10" s="23">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+      <c r="C10" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="D10" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="E10" s="22">
+        <v>2</v>
+      </c>
+      <c r="F10" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="G10" s="22">
+        <f>SUM($E$2:E10)/$E$23</f>
+        <v>0.6</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A11" s="4">
+        <f>A10</f>
+        <v>45972</v>
+      </c>
+      <c r="B11" s="23">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+      <c r="C11" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="E11" s="22">
+        <v>2</v>
+      </c>
+      <c r="F11" s="26" t="s">
+        <v>19</v>
+      </c>
+      <c r="G11" s="22">
+        <f>SUM($E$2:E11)/$E$23</f>
+        <v>0.66666666666666663</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A12" s="4">
+        <f>A11+7</f>
+        <v>45979</v>
+      </c>
+      <c r="B12" s="23">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+      <c r="C12" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="D12" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="F12" s="25"/>
+      <c r="G12" s="1">
+        <f>SUM($E$2:E12)/$E$23</f>
+        <v>0.66666666666666663</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A13" s="4">
+        <f>A12</f>
+        <v>45979</v>
+      </c>
+      <c r="B13" s="23">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+      <c r="C13" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="D13" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="E13" s="22">
+        <v>2</v>
+      </c>
+      <c r="F13" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="G13" s="22">
+        <f>SUM($E$2:E13)/$E$23</f>
+        <v>0.73333333333333328</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A14" s="4">
+        <f>A13+7</f>
+        <v>45986</v>
+      </c>
+      <c r="B14" s="23">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+      <c r="C14" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="D14" s="14" t="s">
+        <v>22</v>
+      </c>
+      <c r="E14" s="22">
+        <v>2</v>
+      </c>
+      <c r="F14" s="27" t="s">
+        <v>23</v>
+      </c>
+      <c r="G14" s="22">
+        <f>SUM($E$2:E14)/$E$23</f>
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A15" s="4">
+        <f>A14</f>
+        <v>45986</v>
+      </c>
+      <c r="B15" s="23">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+      <c r="C15" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="D15" s="14" t="s">
+        <v>22</v>
+      </c>
+      <c r="E15" s="22">
+        <v>2</v>
+      </c>
+      <c r="F15" s="27"/>
+      <c r="G15" s="22">
+        <f>SUM($E$2:E15)/$E$23</f>
+        <v>0.8666666666666667</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A16" s="4">
+        <f>A15+7</f>
+        <v>45993</v>
+      </c>
+      <c r="B16" s="23">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+      <c r="C16" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="D16" s="14" t="s">
+        <v>22</v>
+      </c>
+      <c r="E16" s="22">
+        <v>2</v>
+      </c>
+      <c r="F16" s="27" t="s">
+        <v>25</v>
+      </c>
+      <c r="G16" s="22">
+        <f>SUM($E$2:E16)/$E$23</f>
+        <v>0.93333333333333335</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A17" s="4">
+        <f>A16</f>
+        <v>45993</v>
+      </c>
+      <c r="B17" s="23">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+      <c r="C17" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="D17" s="14" t="s">
+        <v>22</v>
+      </c>
+      <c r="E17" s="22">
+        <v>2</v>
+      </c>
+      <c r="F17" s="27"/>
+      <c r="G17" s="22">
+        <f>SUM($E$2:E17)/$E$23</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="4">
+        <f>A17+7</f>
+        <v>46000</v>
+      </c>
+      <c r="B18" s="23">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+      <c r="C18" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="G18" s="22">
+        <f>SUM($E$2:E18)/$E$23</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="4">
+        <f>A18</f>
+        <v>46000</v>
+      </c>
+      <c r="B19" s="23">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+      <c r="C19" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="D19" s="3"/>
+      <c r="G19" s="22">
+        <f>SUM($E$2:E19)/$E$23</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="4">
+        <f>A19+7</f>
+        <v>46007</v>
+      </c>
+      <c r="B20" s="23">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+      <c r="C20" s="7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A21" s="4">
+        <f>A20</f>
+        <v>46007</v>
+      </c>
+      <c r="B21" s="23">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+      <c r="C21" s="7" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="D22" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="E22" s="2">
+        <f>SUM(E2:E21)</f>
+        <v>30</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="D23" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="E23" s="1">
+        <v>30</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="F14:F15"/>
+    <mergeCell ref="F16:F17"/>
+  </mergeCells>
+  <conditionalFormatting sqref="A1:A1048576">
+    <cfRule type="colorScale" priority="1">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F1 E23 D23:D1048576 D19 D1:D17">
+    <cfRule type="cellIs" dxfId="3" priority="2" operator="equal">
+      <formula>"Theory"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967293" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F1FA0065-A3C8-4E4D-B5EC-36CCF9E12688}">
   <dimension ref="A1:J32"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="10.81640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.77734375" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="9" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="17.7265625" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="6.7265625" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="8.26953125" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="66.81640625" style="13" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.7265625" style="1" hidden="1" customWidth="1"/>
-    <col min="8" max="8" width="24.453125" style="9" hidden="1" customWidth="1"/>
-    <col min="9" max="9" width="5.26953125" hidden="1" customWidth="1"/>
+    <col min="3" max="3" width="17.77734375" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="6.77734375" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="8.21875" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="66.77734375" style="13" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.77734375" style="1" hidden="1" customWidth="1"/>
+    <col min="8" max="8" width="24.44140625" style="9" hidden="1" customWidth="1"/>
+    <col min="9" max="9" width="5.21875" hidden="1" customWidth="1"/>
     <col min="10" max="10" width="0" hidden="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -1369,7 +1935,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A2" s="4">
         <v>45580</v>
       </c>
@@ -1400,7 +1966,7 @@
         <v>6.6666666666666666E-2</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A3" s="4">
         <f>A2</f>
         <v>45580</v>
@@ -1435,7 +2001,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A4" s="4">
         <f>A3+7</f>
         <v>45587</v>
@@ -1470,7 +2036,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A5" s="4">
         <f>A3+8</f>
         <v>45588</v>
@@ -1505,7 +2071,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A6" s="4">
         <v>45601</v>
       </c>
@@ -1539,7 +2105,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A7" s="4">
         <f>A6</f>
         <v>45601</v>
@@ -1571,7 +2137,7 @@
         <v>0.43333333333333335</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A8" s="4">
         <f>A7+7</f>
         <v>45608</v>
@@ -1603,7 +2169,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A9" s="4">
         <f>A8</f>
         <v>45608</v>
@@ -1638,7 +2204,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A10" s="4">
         <f>A9+7</f>
         <v>45615</v>
@@ -1673,7 +2239,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A11" s="4">
         <f>A10</f>
         <v>45615</v>
@@ -1705,7 +2271,7 @@
         <v>0.7</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A12" s="4">
         <f>A11+7</f>
         <v>45622</v>
@@ -1737,7 +2303,7 @@
         <v>0.76666666666666672</v>
       </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A13" s="4">
         <f>A12</f>
         <v>45622</v>
@@ -1767,7 +2333,7 @@
         <v>0.83333333333333337</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A14" s="4">
         <f>A13+7</f>
         <v>45629</v>
@@ -1802,7 +2368,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A15" s="4">
         <f>A14</f>
         <v>45629</v>
@@ -1833,7 +2399,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A16" s="4">
         <f>A15+7</f>
         <v>45636</v>
@@ -1860,7 +2426,7 @@
         <v>1.0333333333333334</v>
       </c>
     </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A17" s="4">
         <f>A16</f>
         <v>45636</v>
@@ -1890,7 +2456,7 @@
         <v>1.0333333333333334</v>
       </c>
     </row>
-    <row r="18" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A18" s="4">
         <f>A17+7</f>
         <v>45643</v>
@@ -1915,7 +2481,7 @@
         <v>1.0333333333333334</v>
       </c>
     </row>
-    <row r="19" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A19" s="4">
         <f>A18</f>
         <v>45643</v>
@@ -1940,7 +2506,7 @@
         <v>1.0333333333333334</v>
       </c>
     </row>
-    <row r="20" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A20" s="4">
         <f>A19+7</f>
         <v>45650</v>
@@ -1959,7 +2525,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="21" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A21" s="4">
         <f>A20</f>
         <v>45650</v>
@@ -1978,7 +2544,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:9" x14ac:dyDescent="0.3">
       <c r="D22" s="1" t="s">
         <v>26</v>
       </c>
@@ -1987,7 +2553,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:9" x14ac:dyDescent="0.3">
       <c r="D23" s="1" t="s">
         <v>27</v>
       </c>
@@ -1995,7 +2561,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:9" x14ac:dyDescent="0.3">
       <c r="E32" s="24"/>
     </row>
   </sheetData>
@@ -2016,7 +2582,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F1 D1:D15 D17:D19 E23 D23:D1048576">
-    <cfRule type="cellIs" dxfId="1" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="2" priority="2" operator="equal">
       <formula>"Theory"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -2028,22 +2594,22 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:H18"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="11" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="4.26953125" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="4.21875" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="18" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="7.26953125" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="8.7265625" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="52.7265625" style="1" customWidth="1"/>
-    <col min="7" max="7" width="9.26953125" style="9"/>
+    <col min="4" max="4" width="7.21875" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="8.77734375" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="52.77734375" style="1" customWidth="1"/>
+    <col min="7" max="7" width="9.21875" style="9"/>
     <col min="8" max="8" width="0" hidden="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -2069,7 +2635,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A2" s="4">
         <v>44860</v>
       </c>
@@ -2097,7 +2663,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" s="4">
         <v>44860</v>
       </c>
@@ -2121,7 +2687,7 @@
       </c>
       <c r="H3" s="30"/>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A4" s="4">
         <v>44867</v>
       </c>
@@ -2147,7 +2713,7 @@
       </c>
       <c r="H4" s="1"/>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A5" s="4">
         <v>44867</v>
       </c>
@@ -2175,7 +2741,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6" s="4">
         <v>44874</v>
       </c>
@@ -2201,7 +2767,7 @@
       </c>
       <c r="H6" s="1"/>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A7" s="4">
         <v>44874</v>
       </c>
@@ -2229,7 +2795,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A8" s="4">
         <v>44881</v>
       </c>
@@ -2255,7 +2821,7 @@
       </c>
       <c r="H8" s="1"/>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A9" s="4">
         <v>44881</v>
       </c>
@@ -2283,7 +2849,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A10" s="4">
         <v>44888</v>
       </c>
@@ -2308,7 +2874,7 @@
       </c>
       <c r="H10" s="1"/>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A11" s="4">
         <v>44888</v>
       </c>
@@ -2333,7 +2899,7 @@
       </c>
       <c r="H11" s="1"/>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A12" s="4">
         <v>44893</v>
       </c>
@@ -2359,7 +2925,7 @@
       </c>
       <c r="H12" s="1"/>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A13" s="4">
         <v>44895</v>
       </c>
@@ -2383,7 +2949,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A14" s="4">
         <v>44895</v>
       </c>
@@ -2405,7 +2971,7 @@
       </c>
       <c r="H14" s="1"/>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A15" s="4">
         <v>44900</v>
       </c>
@@ -2431,7 +2997,7 @@
       </c>
       <c r="H15" s="1"/>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A16" s="4">
         <v>44902</v>
       </c>
@@ -2457,7 +3023,7 @@
       </c>
       <c r="H16" s="1"/>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A17" s="4">
         <v>44907</v>
       </c>
@@ -2483,7 +3049,7 @@
       </c>
       <c r="H17" s="1"/>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
       <c r="C18" s="5" t="s">
         <v>70</v>
       </c>
@@ -2512,7 +3078,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D1:D1048576">
-    <cfRule type="cellIs" dxfId="0" priority="4" operator="equal">
+    <cfRule type="cellIs" dxfId="1" priority="4" operator="equal">
       <formula>"Theory"</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
chore: working on the program
</commit_message>
<xml_diff>
--- a/Program.xlsx
+++ b/Program.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24334"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\repos\teaching\AA2627-unibo-bdcp\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\matte\Downloads\repos\aa2627-unibo-bdcp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{381DDD00-04AD-4F57-A676-0CBE0266AA8F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30F57EB9-E896-4348-AE83-57BD45903BA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="-96" windowWidth="46272" windowHeight="25392" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="38280" yWindow="-240" windowWidth="38640" windowHeight="21840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="AA2627" sheetId="4" r:id="rId1"/>
@@ -32,15 +32,12 @@
         <xcalcf:feature name="microsoft.com:LET_WF"/>
       </xcalcf:calcFeatures>
     </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
-    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="281" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="283" uniqueCount="82">
   <si>
     <t>When</t>
   </si>
@@ -261,16 +258,31 @@
     <t>Introduction, (Towards) Data Platforms (until DWH)</t>
   </si>
   <si>
-    <t>Festa</t>
-  </si>
-  <si>
     <t>Seminar: Technogym?</t>
   </si>
   <si>
     <t>Seminar: Lisa Mazzini?</t>
   </si>
   <si>
-    <t>Data Platforms, Data Governance (beginning of exercise on data profiling)</t>
+    <t>Data Platforms, Data Governance (beginning of exercise on schema ext)</t>
+  </si>
+  <si>
+    <t>Data Governance (until case study on ML + metadata)</t>
+  </si>
+  <si>
+    <t>Holiday</t>
+  </si>
+  <si>
+    <t>Data Governance (until hera seminar)</t>
+  </si>
+  <si>
+    <t>Data Governance (demo LLM wiki?)</t>
+  </si>
+  <si>
+    <t>Cloud Computing (until why moving to the cloud?)</t>
+  </si>
+  <si>
+    <t>Cloud (Migration)</t>
   </si>
 </sst>
 </file>
@@ -401,7 +413,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -476,14 +488,8 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -826,7 +832,7 @@
     <col min="4" max="4" width="6.77734375" style="1" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="8.21875" style="1" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="66.77734375" style="13" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="5.21875" customWidth="1"/>
+    <col min="7" max="7" width="5.21875" hidden="1" customWidth="1"/>
     <col min="8" max="8" width="8.77734375" customWidth="1"/>
   </cols>
   <sheetData>
@@ -892,13 +898,13 @@
       <c r="D3" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="E3" s="28">
-        <v>2</v>
-      </c>
-      <c r="F3" s="29" t="s">
+      <c r="E3" s="1">
+        <v>2</v>
+      </c>
+      <c r="F3" s="27" t="s">
         <v>72</v>
       </c>
-      <c r="G3" s="28">
+      <c r="G3" s="1">
         <f>SUM($E$2:E3)/$E$23</f>
         <v>0.13333333333333333</v>
       </c>
@@ -918,13 +924,13 @@
       <c r="D4" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="E4" s="28">
-        <v>2</v>
-      </c>
-      <c r="F4" s="29" t="s">
-        <v>76</v>
-      </c>
-      <c r="G4" s="28">
+      <c r="E4" s="1">
+        <v>2</v>
+      </c>
+      <c r="F4" s="27" t="s">
+        <v>75</v>
+      </c>
+      <c r="G4" s="1">
         <f>SUM($E$2:E4)/$E$23</f>
         <v>0.2</v>
       </c>
@@ -945,20 +951,20 @@
       <c r="D5" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="E5" s="28">
-        <v>2</v>
-      </c>
-      <c r="F5" s="25" t="s">
-        <v>13</v>
-      </c>
-      <c r="G5" s="28">
+      <c r="E5" s="1">
+        <v>2</v>
+      </c>
+      <c r="F5" s="27" t="s">
+        <v>76</v>
+      </c>
+      <c r="G5" s="1">
         <f>SUM($E$2:E5)/$E$23</f>
         <v>0.26666666666666666</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6" s="4">
-        <f t="shared" ref="A6:A19" si="1">A4+7</f>
+        <f t="shared" ref="A6:A21" si="1">A4+7</f>
         <v>45956</v>
       </c>
       <c r="B6" s="23">
@@ -971,13 +977,13 @@
       <c r="D6" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="E6" s="28">
+      <c r="E6" s="1">
         <v>2</v>
       </c>
       <c r="F6" s="25" t="s">
-        <v>15</v>
-      </c>
-      <c r="G6" s="28">
+        <v>78</v>
+      </c>
+      <c r="G6" s="1">
         <f>SUM($E$2:E6)/$E$23</f>
         <v>0.33333333333333331</v>
       </c>
@@ -997,13 +1003,13 @@
       <c r="D7" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="E7" s="28">
+      <c r="E7" s="1">
         <v>2</v>
       </c>
       <c r="F7" s="25" t="s">
-        <v>16</v>
-      </c>
-      <c r="G7" s="28">
+        <v>79</v>
+      </c>
+      <c r="G7" s="1">
         <f>SUM($E$2:E7)/$E$23</f>
         <v>0.4</v>
       </c>
@@ -1023,13 +1029,13 @@
       <c r="D8" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="E8" s="28">
+      <c r="E8" s="1">
         <v>2</v>
       </c>
       <c r="F8" s="25" t="s">
-        <v>17</v>
-      </c>
-      <c r="G8" s="28">
+        <v>80</v>
+      </c>
+      <c r="G8" s="1">
         <f>SUM($E$2:E8)/$E$23</f>
         <v>0.46666666666666667</v>
       </c>
@@ -1049,13 +1055,13 @@
       <c r="D9" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="E9" s="28">
+      <c r="E9" s="1">
         <v>2</v>
       </c>
       <c r="F9" s="25" t="s">
-        <v>18</v>
-      </c>
-      <c r="G9" s="28">
+        <v>19</v>
+      </c>
+      <c r="G9" s="1">
         <f>SUM($E$2:E9)/$E$23</f>
         <v>0.53333333333333333</v>
       </c>
@@ -1075,13 +1081,13 @@
       <c r="D10" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="E10" s="28">
+      <c r="E10" s="1">
         <v>2</v>
       </c>
       <c r="F10" s="25" t="s">
-        <v>19</v>
-      </c>
-      <c r="G10" s="28">
+        <v>20</v>
+      </c>
+      <c r="G10" s="1">
         <f>SUM($E$2:E10)/$E$23</f>
         <v>0.6</v>
       </c>
@@ -1101,13 +1107,13 @@
       <c r="D11" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="E11" s="28">
+      <c r="E11" s="1">
         <v>2</v>
       </c>
       <c r="F11" s="25" t="s">
-        <v>20</v>
-      </c>
-      <c r="G11" s="28">
+        <v>19</v>
+      </c>
+      <c r="G11" s="1">
         <f>SUM($E$2:E11)/$E$23</f>
         <v>0.66666666666666663</v>
       </c>
@@ -1127,13 +1133,13 @@
       <c r="D12" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="E12" s="28">
+      <c r="E12" s="1">
         <v>2</v>
       </c>
       <c r="F12" s="25" t="s">
-        <v>19</v>
-      </c>
-      <c r="G12" s="28">
+        <v>21</v>
+      </c>
+      <c r="G12" s="1">
         <f>SUM($E$2:E12)/$E$23</f>
         <v>0.73333333333333328</v>
       </c>
@@ -1153,13 +1159,13 @@
       <c r="D13" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="E13" s="28">
+      <c r="E13" s="1">
         <v>2</v>
       </c>
       <c r="F13" s="25" t="s">
-        <v>21</v>
-      </c>
-      <c r="G13" s="28">
+        <v>81</v>
+      </c>
+      <c r="G13" s="1">
         <f>SUM($E$2:E13)/$E$23</f>
         <v>0.8</v>
       </c>
@@ -1179,13 +1185,15 @@
       <c r="D14" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="E14" s="28">
-        <v>0</v>
-      </c>
-      <c r="F14" s="27"/>
-      <c r="G14" s="28">
+      <c r="E14" s="1">
+        <v>2</v>
+      </c>
+      <c r="F14" s="25" t="s">
+        <v>52</v>
+      </c>
+      <c r="G14" s="1">
         <f>SUM($E$2:E14)/$E$23</f>
-        <v>0.8</v>
+        <v>0.8666666666666667</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.3">
@@ -1203,15 +1211,15 @@
       <c r="D15" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="E15" s="28">
-        <v>2</v>
-      </c>
-      <c r="F15" s="27" t="s">
-        <v>74</v>
-      </c>
-      <c r="G15" s="28">
+      <c r="E15" s="1">
+        <v>2</v>
+      </c>
+      <c r="F15" s="26" t="s">
+        <v>73</v>
+      </c>
+      <c r="G15" s="1">
         <f>SUM($E$2:E15)/$E$23</f>
-        <v>0.8666666666666667</v>
+        <v>0.93333333333333335</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.3">
@@ -1229,13 +1237,15 @@
       <c r="D16" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="E16" s="28">
+      <c r="E16" s="1">
         <v>0</v>
       </c>
-      <c r="F16" s="27"/>
-      <c r="G16" s="28">
+      <c r="F16" s="25" t="s">
+        <v>56</v>
+      </c>
+      <c r="G16" s="1">
         <f>SUM($E$2:E16)/$E$23</f>
-        <v>0.8666666666666667</v>
+        <v>0.93333333333333335</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.3">
@@ -1253,18 +1263,18 @@
       <c r="D17" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="E17" s="28">
-        <v>2</v>
-      </c>
-      <c r="F17" s="27" t="s">
-        <v>75</v>
-      </c>
-      <c r="G17" s="28">
+      <c r="E17" s="1">
+        <v>2</v>
+      </c>
+      <c r="F17" s="26" t="s">
+        <v>74</v>
+      </c>
+      <c r="G17" s="1">
         <f>SUM($E$2:E17)/$E$23</f>
-        <v>0.93333333333333335</v>
-      </c>
-    </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A18" s="4">
         <f t="shared" si="1"/>
         <v>45998</v>
@@ -1274,18 +1284,17 @@
         <v>0</v>
       </c>
       <c r="C18" s="7" t="s">
-        <v>8</v>
+        <v>71</v>
       </c>
       <c r="D18" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="E18" s="28"/>
-      <c r="G18" s="28">
+      <c r="G18" s="1">
         <f>SUM($E$2:E18)/$E$23</f>
-        <v>0.93333333333333335</v>
-      </c>
-    </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A19" s="4">
         <f t="shared" si="1"/>
         <v>45999</v>
@@ -1300,39 +1309,37 @@
       <c r="D19" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="E19" s="28"/>
       <c r="F19" s="13" t="s">
-        <v>73</v>
-      </c>
-      <c r="G19" s="28">
+        <v>77</v>
+      </c>
+      <c r="G19" s="1">
         <f>SUM($E$2:E19)/$E$23</f>
-        <v>0.93333333333333335</v>
-      </c>
-    </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A20" s="4">
-        <f>A19+7</f>
-        <v>46006</v>
+        <f t="shared" si="1"/>
+        <v>46005</v>
       </c>
       <c r="B20" s="23">
         <f t="shared" si="0"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C20" s="7" t="s">
-        <v>8</v>
+        <v>71</v>
       </c>
       <c r="D20" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="E20" s="28"/>
-      <c r="G20" s="28">
+      <c r="G20" s="1">
         <f>SUM($E$2:E20)/$E$23</f>
-        <v>0.93333333333333335</v>
-      </c>
-    </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A21" s="4">
-        <f>A20</f>
+        <f t="shared" si="1"/>
         <v>46006</v>
       </c>
       <c r="B21" s="23">
@@ -1345,22 +1352,21 @@
       <c r="D21" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="E21" s="28"/>
-      <c r="G21" s="28">
+      <c r="G21" s="1">
         <f>SUM($E$2:E21)/$E$23</f>
-        <v>0.93333333333333335</v>
-      </c>
-    </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="D22" s="2" t="s">
         <v>26</v>
       </c>
       <c r="E22" s="2">
         <f>SUM(E2:E21)</f>
-        <v>28</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="D23" s="2" t="s">
         <v>27</v>
       </c>
@@ -1381,13 +1387,13 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F1 E23 D23:D1048576 D1:D17">
-    <cfRule type="cellIs" dxfId="4" priority="3" operator="equal">
+  <conditionalFormatting sqref="D1:D21">
+    <cfRule type="cellIs" dxfId="4" priority="1" operator="equal">
       <formula>"Theory"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D18:D21">
-    <cfRule type="cellIs" dxfId="3" priority="1" operator="equal">
+  <conditionalFormatting sqref="F1 E23 D23:D1048576">
+    <cfRule type="cellIs" dxfId="3" priority="3" operator="equal">
       <formula>"Theory"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -1689,7 +1695,7 @@
       <c r="E11" s="22">
         <v>2</v>
       </c>
-      <c r="F11" s="26" t="s">
+      <c r="F11" s="13" t="s">
         <v>19</v>
       </c>
       <c r="G11" s="22">
@@ -1762,7 +1768,7 @@
       <c r="E14" s="22">
         <v>2</v>
       </c>
-      <c r="F14" s="30" t="s">
+      <c r="F14" s="28" t="s">
         <v>23</v>
       </c>
       <c r="G14" s="22">
@@ -1788,7 +1794,7 @@
       <c r="E15" s="22">
         <v>2</v>
       </c>
-      <c r="F15" s="30"/>
+      <c r="F15" s="28"/>
       <c r="G15" s="22">
         <f>SUM($E$2:E15)/$E$23</f>
         <v>0.8666666666666667</v>
@@ -1812,7 +1818,7 @@
       <c r="E16" s="22">
         <v>2</v>
       </c>
-      <c r="F16" s="30" t="s">
+      <c r="F16" s="28" t="s">
         <v>25</v>
       </c>
       <c r="G16" s="22">
@@ -1838,7 +1844,7 @@
       <c r="E17" s="22">
         <v>2</v>
       </c>
-      <c r="F17" s="30"/>
+      <c r="F17" s="28"/>
       <c r="G17" s="22">
         <f>SUM($E$2:E17)/$E$23</f>
         <v>1</v>
@@ -1939,7 +1945,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F1 E23 D23:D1048576 D19 D1:D17">
+  <conditionalFormatting sqref="F1 D1:D17 D19 E23 D23:D1048576">
     <cfRule type="cellIs" dxfId="2" priority="2" operator="equal">
       <formula>"Theory"</formula>
     </cfRule>
@@ -2352,7 +2358,7 @@
       <c r="E12" s="22">
         <v>2</v>
       </c>
-      <c r="F12" s="31" t="s">
+      <c r="F12" s="29" t="s">
         <v>50</v>
       </c>
       <c r="G12" s="17">
@@ -2384,7 +2390,7 @@
       <c r="E13" s="22">
         <v>2</v>
       </c>
-      <c r="F13" s="31"/>
+      <c r="F13" s="29"/>
       <c r="G13" s="17">
         <v>2</v>
       </c>
@@ -2414,7 +2420,7 @@
       <c r="E14" s="22">
         <v>2</v>
       </c>
-      <c r="F14" s="31" t="s">
+      <c r="F14" s="29" t="s">
         <v>53</v>
       </c>
       <c r="G14" s="17">
@@ -2449,7 +2455,7 @@
       <c r="E15" s="22">
         <v>2</v>
       </c>
-      <c r="F15" s="31"/>
+      <c r="F15" s="29"/>
       <c r="G15" s="1" t="s">
         <v>56</v>
       </c>
@@ -2715,14 +2721,14 @@
       <c r="E2" s="1">
         <v>2</v>
       </c>
-      <c r="F2" s="32" t="s">
+      <c r="F2" s="30" t="s">
         <v>30</v>
       </c>
       <c r="G2" s="10">
         <f>SUM($E$2:E2)/$E$18</f>
         <v>6.6666666666666666E-2</v>
       </c>
-      <c r="H2" s="33" t="s">
+      <c r="H2" s="31" t="s">
         <v>60</v>
       </c>
     </row>
@@ -2743,12 +2749,12 @@
       <c r="E3" s="1">
         <v>2</v>
       </c>
-      <c r="F3" s="32"/>
+      <c r="F3" s="30"/>
       <c r="G3" s="10">
         <f>SUM($E$2:E3)/$E$18</f>
         <v>0.13333333333333333</v>
       </c>
-      <c r="H3" s="33"/>
+      <c r="H3" s="31"/>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A4" s="4">

</xml_diff>

<commit_message>
fix: update labs and layouts
</commit_message>
<xml_diff>
--- a/Program.xlsx
+++ b/Program.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24334"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\matte\Downloads\repos\aa2627-unibo-bdcp\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\repos\teaching\AA2627-unibo-bdcp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30F57EB9-E896-4348-AE83-57BD45903BA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7709AE0-6CA6-4954-99EE-4508CA0155A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="-240" windowWidth="38640" windowHeight="21840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="46296" windowHeight="25416" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="AA2627" sheetId="4" r:id="rId1"/>
@@ -32,6 +32,9 @@
         <xcalcf:feature name="microsoft.com:LET_WF"/>
       </xcalcf:calcFeatures>
     </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
   </extLst>
 </workbook>
 </file>
@@ -273,9 +276,6 @@
     <t>Holiday</t>
   </si>
   <si>
-    <t>Data Governance (until hera seminar)</t>
-  </si>
-  <si>
     <t>Data Governance (demo LLM wiki?)</t>
   </si>
   <si>
@@ -283,6 +283,9 @@
   </si>
   <si>
     <t>Cloud (Migration)</t>
+  </si>
+  <si>
+    <t>Data Governance (until hera seminar?)</t>
   </si>
 </sst>
 </file>
@@ -413,7 +416,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -505,6 +508,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -980,8 +986,8 @@
       <c r="E6" s="1">
         <v>2</v>
       </c>
-      <c r="F6" s="25" t="s">
-        <v>78</v>
+      <c r="F6" s="32" t="s">
+        <v>81</v>
       </c>
       <c r="G6" s="1">
         <f>SUM($E$2:E6)/$E$23</f>
@@ -1007,7 +1013,7 @@
         <v>2</v>
       </c>
       <c r="F7" s="25" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="G7" s="1">
         <f>SUM($E$2:E7)/$E$23</f>
@@ -1033,7 +1039,7 @@
         <v>2</v>
       </c>
       <c r="F8" s="25" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="G8" s="1">
         <f>SUM($E$2:E8)/$E$23</f>
@@ -1163,7 +1169,7 @@
         <v>2</v>
       </c>
       <c r="F13" s="25" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="G13" s="1">
         <f>SUM($E$2:E13)/$E$23</f>

</xml_diff>